<commit_message>
fix(core-beta): block missing run-owned experts safely
</commit_message>
<xml_diff>
--- a/PRD/QBot完整生产灰度门禁Casebook_184条_2026-08-03.xlsx
+++ b/PRD/QBot完整生产灰度门禁Casebook_184条_2026-08-03.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心内测Case" sheetId="1" r:id="Re665fbfffbdc4fca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设计总览" sheetId="2" r:id="R3d62d7a5010b4dc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="覆盖矩阵" sheetId="3" r:id="R6d94f574c90e4a8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="执行配置" sheetId="4" r:id="R1b751970ed3546c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据与断言" sheetId="5" r:id="R14ff78434fe74d5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="旧Case审计" sheetId="6" r:id="R58e67be65d4e41c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="旧Case收敛映射" sheetId="7" r:id="Re116e597f7914a22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MR与源码设计依据" sheetId="8" r:id="R3e237dba0d5c4813"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="生产灰度准入" sheetId="9" r:id="R6fc5929e9d2e48da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整功能门禁" sheetId="10" r:id="R386f94b2b42b4e94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整门禁源码依据" sheetId="11" r:id="R1a775462d02d4275"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心内测Case" sheetId="1" r:id="R09b2cfbd1e044606"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设计总览" sheetId="2" r:id="R245548b6e7024e11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="覆盖矩阵" sheetId="3" r:id="Rabbc182b0f064845"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="执行配置" sheetId="4" r:id="R15d28c3071194118"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据与断言" sheetId="5" r:id="Rbd2474a491364cbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="旧Case审计" sheetId="6" r:id="Re0008719302246f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="旧Case收敛映射" sheetId="7" r:id="Rf6afc74b51cd4895"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MR与源码设计依据" sheetId="8" r:id="R5dea89455f1c491a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="生产灰度准入" sheetId="9" r:id="R36a6b8efe0dd4d85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整功能门禁" sheetId="10" r:id="Rc046694c4c6c4447"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整门禁源码依据" sheetId="11" r:id="Ra2e5e5a30b36414a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7097,7 +7097,7 @@
         <x:v>BETA-EXPERT-002/007产出的研究专家已发布；依赖可用。</x:v>
       </x:c>
       <x:c r="J53" s="48" t="str">
-        <x:v>选择一个当天可验证的产品/行业问题；要求至少两个官方来源。</x:v>
+        <x:v>固定研究主题：截至2026-08-06，OpenAI Responses API 与 Chat Completions API 的官方定位、主要能力差异和迁移建议；要求至少两个可打开的 OpenAI 官方来源。</x:v>
       </x:c>
       <x:c r="K53" s="48" t="str">
         <x:v>1. 从专家详情召唤研究专家并核对exact release identity
@@ -7138,7 +7138,7 @@
         <x:v>[{"number":1,"action_id":"beta-expert-008-prepare","operation":"prepare","target":"BETA-EXPERT-008:prepare","declared_step":"按前置条件执行初始化、清理并校验fixture；原始步骤：从专家详情召唤研究专家并核对exact release identity","command":"prepare_expert_use","executor":"core-beta/scenario/beta-expert-008/v1","expected_state":"页面、发布身份、账号、fixture与执行策略全部ready","evidence_roles":["before_screenshot","action_receipt","after_screenshot"],"assertions":[{"id":"page-ready","path":"state.page.body_text_length","operator":"gte","expected":1}]},{"number":2,"action_id":"beta-expert-008-execute","operation":"execute","target":"BETA-EXPERT-008:execute","declared_step":"1. 从专家详情召唤研究专家并核对exact release identity；2. 完成检索和来源比较两轮，保存tools/call与来源；3. 第三轮形成带引用结论并核对最近召唤与task pin","command":"execute_expert_use","executor":"core-beta/scenario/beta-expert-008/v1","expected_state":"全部声明操作由对应真实UI/bridge/composer handler执行并生成动作回执","evidence_roles":["before_screenshot","action_receipt","after_screenshot"],"assertions":[{"id":"observable-assertion","path":"receipt.assertion_count","operator":"gte","expected":1}]},{"number":3,"action_id":"beta-expert-008-verify","operation":"verify","target":"BETA-EXPERT-008:verify","declared_step":"按taskId、能力identity、公开状态、完整回复、产物内容和负向边界执行精准断言与清理读回","command":"verify_expert_use","executor":"core-beta/scenario/beta-expert-008/v1","expected_state":"精准断言无失败且证据角色可生成不可变manifest","evidence_roles":["before_screenshot","action_receipt","after_screenshot"],"assertions":[{"id":"no-step-failure","path":"receipt.step_failures","operator":"equals","expected":0},{"id":"no-assertion-failure","path":"receipt.assertion_failures","operator":"equals","expected":0}]}]</x:v>
       </x:c>
       <x:c r="W53" s="48" t="str">
-        <x:v>[{"turn":1,"prompt":"检索两个官方来源说明目标问题现状。","oracle":"回复完整、与当前task及能力身份一致，并满足本Case精准断言","must_not_include":["traceback","DEEPBANK_","apiKey","Authorization: Bearer"]},{"turn":2,"prompt":"比较两份来源的共识、冲突和时效性。","oracle":"回复完整、与当前task及能力身份一致，并满足本Case精准断言","must_not_include":["traceback","DEEPBANK_","apiKey","Authorization: Bearer"]},{"turn":3,"prompt":"给出带引用的结论、风险和下一步。","oracle":"回复完整、与当前task及能力身份一致，并满足本Case精准断言","must_not_include":["traceback","DEEPBANK_","apiKey","Authorization: Bearer"]}]</x:v>
+        <x:v>[{"turn":1,"prompt":"检索至少两个 OpenAI 官方来源，说明截至2026-08-06 Responses API 与 Chat Completions API 的官方定位、主要能力差异和迁移建议；每个来源给出标题、日期或更新时间（如页面提供）及可打开 URL。","oracle":"回复完整、与当前task及能力身份一致，并满足本Case精准断言","must_not_include":["traceback","DEEPBANK_","apiKey","Authorization: Bearer"]},{"turn":2,"prompt":"仅基于上一轮的 OpenAI 官方来源，比较两者在工具能力、会话状态和迁移路径上的共识、差异与时效性，不得引入未引用来源。","oracle":"回复完整、与当前task及能力身份一致，并满足本Case精准断言","must_not_include":["traceback","DEEPBANK_","apiKey","Authorization: Bearer"]},{"turn":3,"prompt":"基于上述官方来源给出是否应优先迁移到 Responses API 的带引用结论、风险和下一步；逐条引用可打开 URL，并标明截至2026-08-06。","oracle":"回复完整、与当前task及能力身份一致，并满足本Case精准断言","must_not_include":["traceback","DEEPBANK_","apiKey","Authorization: Bearer"]}]</x:v>
       </x:c>
       <x:c r="X53" s="48"/>
       <x:c r="Y53" s="48" t="str">

</xml_diff>